<commit_message>
Update 7 terms in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -15912,7 +15912,7 @@
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Symptom severity that is associated with a depression symtom.</t>
+          <t>Symptom severity that is associated with a depression symptom.</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
@@ -16113,7 +16113,7 @@
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Symptom severity that is associated with a depression symtom.</t>
+          <t>Symptom severity that is associated with a depression symptom.</t>
         </is>
       </c>
       <c r="J237" t="inlineStr">
@@ -16314,7 +16314,7 @@
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Symptom severity that is associated with a depression symtom.</t>
+          <t>Symptom severity that is associated with a depression symptom.</t>
         </is>
       </c>
       <c r="J240" t="inlineStr">
@@ -16577,7 +16577,7 @@
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Symptom severity that is associated with a depression symtom.</t>
+          <t>Symptom severity that is associated with a depression symptom.</t>
         </is>
       </c>
       <c r="J244" t="inlineStr">
@@ -26154,12 +26154,12 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t>number of contact events</t>
+          <t>number of intervention contact events</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>A data item that is the number of contact events in an intervention temporal part.</t>
+          <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
@@ -31305,7 +31305,7 @@
       </c>
       <c r="I508" t="inlineStr">
         <is>
-          <t>Symptom severity that is associated with a depression symtom.</t>
+          <t>Symptom severity that is associated with a depression symptom.</t>
         </is>
       </c>
       <c r="J508" t="inlineStr">
@@ -32637,7 +32637,7 @@
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>Recuperando datos. Espere unos segundos e intente cortar o copiar de nuevo.</t>
+          <t>An adverse event following an intervention in which there is an inability to fall asleep or to stay asleep as long as desired.</t>
         </is>
       </c>
       <c r="J529" t="inlineStr">

</xml_diff>